<commit_message>
import characters & animation
</commit_message>
<xml_diff>
--- a/eoe/Assets/Excels/HeroConfig.xlsx
+++ b/eoe/Assets/Excels/HeroConfig.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="16">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -67,19 +67,7 @@
     <t xml:space="preserve">gold</t>
   </si>
   <si>
-    <t xml:space="preserve">hero.101</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hero.102</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hero.103</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hero.104</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hero.105</t>
+    <t xml:space="preserve">Milo</t>
   </si>
 </sst>
 </file>
@@ -471,7 +459,7 @@
         <v>102</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C3" s="1" t="n">
         <v>2002</v>
@@ -518,7 +506,7 @@
         <v>103</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C4" s="1" t="n">
         <v>2003</v>
@@ -565,7 +553,7 @@
         <v>104</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C5" s="1" t="n">
         <v>2004</v>
@@ -612,7 +600,7 @@
         <v>105</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C6" s="1" t="n">
         <v>2005</v>

</xml_diff>

<commit_message>
refactor: remove unused hero ultimate config
</commit_message>
<xml_diff>
--- a/eoe/Assets/Excels/HeroConfig.xlsx
+++ b/eoe/Assets/Excels/HeroConfig.xlsx
@@ -344,7 +344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.5" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="15.63" customWidth="1" style="2" min="1" max="1"/>
@@ -379,55 +379,50 @@
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>ultimateId</t>
+          <t>health</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>attack</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>attack</t>
+          <t>attackRange</t>
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>attackRange</t>
+          <t>attackSpeed</t>
         </is>
       </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
-          <t>attackSpeed</t>
+          <t>critChance</t>
         </is>
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>critChance</t>
+          <t>critDamage</t>
         </is>
       </c>
       <c r="K1" s="2" t="inlineStr">
         <is>
-          <t>critDamage</t>
+          <t>lifesteal</t>
         </is>
       </c>
       <c r="L1" s="2" t="inlineStr">
         <is>
-          <t>lifesteal</t>
+          <t>skillCooldown</t>
         </is>
       </c>
       <c r="M1" s="2" t="inlineStr">
         <is>
-          <t>skillCooldown</t>
+          <t>expMultiplier</t>
         </is>
       </c>
       <c r="N1" s="2" t="inlineStr">
-        <is>
-          <t>expMultiplier</t>
-        </is>
-      </c>
-      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>gold</t>
         </is>
@@ -435,7 +430,7 @@
     </row>
     <row r="2" ht="16.5" customHeight="1" s="3">
       <c r="A2" s="2" t="n">
-        <v>101</v>
+        <v>1001</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
@@ -443,56 +438,53 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>2011</v>
+        <v>1101</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>2001</v>
+        <v>0</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>2001</v>
+        <v>20</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="G2" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N2" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H2" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="I2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J2" s="2" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="K2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="N2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O2" s="2" t="n">
-        <v>5</v>
-      </c>
     </row>
     <row r="3" ht="16.5" customHeight="1" s="3">
-      <c r="O3" s="2" t="n"/>
+      <c r="N3" s="2" t="n"/>
     </row>
     <row r="4" ht="16.5" customHeight="1" s="3">
-      <c r="O4" s="2" t="n"/>
+      <c r="N4" s="2" t="n"/>
     </row>
     <row r="5" ht="16.5" customHeight="1" s="3">
-      <c r="O5" s="2" t="n"/>
+      <c r="N5" s="2" t="n"/>
     </row>
     <row r="6" ht="16.5" customHeight="1" s="3">
-      <c r="O6" s="2" t="n"/>
+      <c r="N6" s="2" t="n"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>